<commit_message>
Update ponentes emails for Jorge Hoyos, Erika Betancourt, Katherine Santiana and add Apps Script review flow for Erika
</commit_message>
<xml_diff>
--- a/piloto_envio_ponentes.xlsx
+++ b/piloto_envio_ponentes.xlsx
@@ -737,7 +737,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>[PENDIENTE - NO SUMINISTRADO]</t>
+          <t>jorgehhoyos@gmail.com</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>[PENDIENTE - NO SUMINISTRADO]</t>
+          <t>erbetancourt@utp.edu.co</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>[PENDIENTE - NO SUMINISTRADO]</t>
+          <t>ksantiana@bolivariano.edu.ec</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Remove recording link from email template and adjust subject line to focus exclusively on official certificate
</commit_message>
<xml_diff>
--- a/piloto_envio_ponentes.xlsx
+++ b/piloto_envio_ponentes.xlsx
@@ -618,7 +618,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Certificado Oficial de Ponente y Grabación - II Foro de Editores de Revistas Científicas 2026</t>
+          <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Certificado Oficial de Ponente y Grabación - II Foro de Editores de Revistas Científicas 2026</t>
+          <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Certificado Oficial de Ponente y Grabación - II Foro de Editores de Revistas Científicas 2026</t>
+          <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Certificado Oficial de Ponente y Grabación - II Foro de Editores de Revistas Científicas 2026</t>
+          <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Certificado Oficial de Ponente y Grabación - II Foro de Editores de Revistas Científicas 2026</t>
+          <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Certificado Oficial de Ponente y Grabación - II Foro de Editores de Revistas Científicas 2026</t>
+          <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Certificado Oficial de Ponente y Grabación - II Foro de Editores de Revistas Científicas 2026</t>
+          <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Certificado Oficial de Ponente y Grabación - II Foro de Editores de Revistas Científicas 2026</t>
+          <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Certificado Oficial de Ponente y Grabación - II Foro de Editores de Revistas Científicas 2026</t>
+          <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Certificado Oficial de Ponente y Grabación - II Foro de Editores de Revistas Científicas 2026</t>
+          <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>Certificado Oficial de Ponente y Grabación - II Foro de Editores de Revistas Científicas 2026</t>
+          <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Certificado Oficial de Ponente y Grabación - II Foro de Editores de Revistas Científicas 2026</t>
+          <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Migrate Leandro Ceballos to Ponente FORO26-PON-013, renumber asistentes, update pilot and master Excels with revision and definitive modes
</commit_message>
<xml_diff>
--- a/piloto_envio_ponentes.xlsx
+++ b/piloto_envio_ponentes.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -491,11 +491,10 @@
     <col width="35" customWidth="1" min="7" max="7"/>
     <col width="45" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="35" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -556,15 +555,10 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Enlace Grabación (Stream)</t>
+          <t>Archivo PDF Local</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Archivo PDF Local</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Estado Envío</t>
         </is>
@@ -628,15 +622,10 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>https://uniminuto0-my.sharepoint.com/personal/felix_duenas_uniminuto_edu/_layouts/15/stream.aspx?id=%2Fpersonal%2Ffelix%5Fduenas%5Funiminuto%5Fedu%2FDocuments%2FGrabaciones%2FII%20FORO%20DE%20EDITORES%20DE%20REVISTAS%20CIENT%C3%8DFICAS%2D20260911%5F080635%2DGrabaci%C3%B3n%20de%20la%20reuni%C3%B3n%2Emp4&amp;ga=1&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E692c7bc5%2Df83b%2D4dbf%2D905d%2D7cb360d59b9e</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
           <t>certificados/ponentes/certificado - Nohelia Yaneth Alfonzo Villegas.pdf</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
@@ -700,87 +689,77 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>https://uniminuto0-my.sharepoint.com/personal/felix_duenas_uniminuto_edu/_layouts/15/stream.aspx?id=%2Fpersonal%2Ffelix%5Fduenas%5Funiminuto%5Fedu%2FDocuments%2FGrabaciones%2FII%20FORO%20DE%20EDITORES%20DE%20REVISTAS%20CIENT%C3%8DFICAS%2D20260911%5F080635%2DGrabaci%C3%B3n%20de%20la%20reuni%C3%B3n%2Emp4&amp;ga=1&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E692c7bc5%2Df83b%2D4dbf%2D905d%2D7cb360d59b9e</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
           <t>certificados/ponentes/certificado - Zahira Felicidad Silano Higuera.pdf</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>FORO26-PON-003</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Jorge Hernán Hoyos Rentería</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Estimado Jorge Hernán Hoyos Rentería</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>juan.nieto2@utp.edu.co</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>jorgehhoyos@gmail.com</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>[NO REGISTRADO EN PROGRAMA]</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Revista Saber Ser</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>ApaWizard: automatización editorial para fortalecer la publicación digital, el acceso abierto y la producción XML/JATS en revistas académicas</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Visibilidad científica y mundo digital</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>https://juannietoval.github.io/certificaci-n-II-foro/?id=FORO26-PON-003</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
-        <is>
-          <t>https://uniminuto0-my.sharepoint.com/personal/felix_duenas_uniminuto_edu/_layouts/15/stream.aspx?id=%2Fpersonal%2Ffelix%5Fduenas%5Funiminuto%5Fedu%2FDocuments%2FGrabaciones%2FII%20FORO%20DE%20EDITORES%20DE%20REVISTAS%20CIENT%C3%8DFICAS%2D20260911%5F080635%2DGrabaci%C3%B3n%20de%20la%20reuni%C3%B3n%2Emp4&amp;ga=1&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E692c7bc5%2Df83b%2D4dbf%2D905d%2D7cb360d59b9e</t>
-        </is>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>certificados/ponentes/certificado - Jorge Hernán Hoyos Rentería.pdf</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
@@ -844,15 +823,10 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>https://uniminuto0-my.sharepoint.com/personal/felix_duenas_uniminuto_edu/_layouts/15/stream.aspx?id=%2Fpersonal%2Ffelix%5Fduenas%5Funiminuto%5Fedu%2FDocuments%2FGrabaciones%2FII%20FORO%20DE%20EDITORES%20DE%20REVISTAS%20CIENT%C3%8DFICAS%2D20260911%5F080635%2DGrabaci%C3%B3n%20de%20la%20reuni%C3%B3n%2Emp4&amp;ga=1&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E692c7bc5%2Df83b%2D4dbf%2D905d%2D7cb360d59b9e</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
           <t>certificados/ponentes/certificado - Fabian Andrey Zarta Rojas.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
@@ -916,87 +890,77 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>https://uniminuto0-my.sharepoint.com/personal/felix_duenas_uniminuto_edu/_layouts/15/stream.aspx?id=%2Fpersonal%2Ffelix%5Fduenas%5Funiminuto%5Fedu%2FDocuments%2FGrabaciones%2FII%20FORO%20DE%20EDITORES%20DE%20REVISTAS%20CIENT%C3%8DFICAS%2D20260911%5F080635%2DGrabaci%C3%B3n%20de%20la%20reuni%C3%B3n%2Emp4&amp;ga=1&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E692c7bc5%2Df83b%2D4dbf%2D905d%2D7cb360d59b9e</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
           <t>certificados/ponentes/certificado - Francisco Javier González Gálvez.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>FORO26-PON-006</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Erika Betancourt</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Estimada Erika Betancourt</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>juan.nieto2@utp.edu.co</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>erbetancourt@utp.edu.co</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>[NO REGISTRADO EN PROGRAMA]</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Universidad Tecnológica de Pereira</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Presentación de la Revista Miradas</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Socialización de Revistas Científicas</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>https://juannietoval.github.io/certificaci-n-II-foro/?id=FORO26-PON-006</t>
         </is>
       </c>
-      <c r="L7" s="5" t="inlineStr">
-        <is>
-          <t>https://uniminuto0-my.sharepoint.com/personal/felix_duenas_uniminuto_edu/_layouts/15/stream.aspx?id=%2Fpersonal%2Ffelix%5Fduenas%5Funiminuto%5Fedu%2FDocuments%2FGrabaciones%2FII%20FORO%20DE%20EDITORES%20DE%20REVISTAS%20CIENT%C3%8DFICAS%2D20260911%5F080635%2DGrabaci%C3%B3n%20de%20la%20reuni%C3%B3n%2Emp4&amp;ga=1&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E692c7bc5%2Df83b%2D4dbf%2D905d%2D7cb360d59b9e</t>
-        </is>
-      </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>certificados/ponentes/certificado - Erika Betancourt.pdf</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
@@ -1060,87 +1024,77 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>https://uniminuto0-my.sharepoint.com/personal/felix_duenas_uniminuto_edu/_layouts/15/stream.aspx?id=%2Fpersonal%2Ffelix%5Fduenas%5Funiminuto%5Fedu%2FDocuments%2FGrabaciones%2FII%20FORO%20DE%20EDITORES%20DE%20REVISTAS%20CIENT%C3%8DFICAS%2D20260911%5F080635%2DGrabaci%C3%B3n%20de%20la%20reuni%C3%B3n%2Emp4&amp;ga=1&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E692c7bc5%2Df83b%2D4dbf%2D905d%2D7cb360d59b9e</t>
-        </is>
-      </c>
-      <c r="M8" s="3" t="inlineStr">
-        <is>
           <t>certificados/ponentes/certificado - Yesenia del Valle Centeno de López.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>FORO26-PON-008</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Katherine Santiana Rosado</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Estimada Katherine Santiana Rosado</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>juan.nieto2@utp.edu.co</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>ksantiana@bolivariano.edu.ec</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>[NO REGISTRADO EN PROGRAMA]</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Instituto Superior Tecnológico Bolivariano de Tecnología</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>La transformación editorial bajo los principios de la ciencia abierta: caso Identidad Bolivariana</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Ética y buenas prácticas editoriales</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>https://juannietoval.github.io/certificaci-n-II-foro/?id=FORO26-PON-008</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
-        <is>
-          <t>https://uniminuto0-my.sharepoint.com/personal/felix_duenas_uniminuto_edu/_layouts/15/stream.aspx?id=%2Fpersonal%2Ffelix%5Fduenas%5Funiminuto%5Fedu%2FDocuments%2FGrabaciones%2FII%20FORO%20DE%20EDITORES%20DE%20REVISTAS%20CIENT%C3%8DFICAS%2D20260911%5F080635%2DGrabaci%C3%B3n%20de%20la%20reuni%C3%B3n%2Emp4&amp;ga=1&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E692c7bc5%2Df83b%2D4dbf%2D905d%2D7cb360d59b9e</t>
-        </is>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="L9" s="3" t="inlineStr">
         <is>
           <t>certificados/ponentes/certificado - Katherine Santiana Rosado.pdf</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
@@ -1204,15 +1158,10 @@
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>https://uniminuto0-my.sharepoint.com/personal/felix_duenas_uniminuto_edu/_layouts/15/stream.aspx?id=%2Fpersonal%2Ffelix%5Fduenas%5Funiminuto%5Fedu%2FDocuments%2FGrabaciones%2FII%20FORO%20DE%20EDITORES%20DE%20REVISTAS%20CIENT%C3%8DFICAS%2D20260911%5F080635%2DGrabaci%C3%B3n%20de%20la%20reuni%C3%B3n%2Emp4&amp;ga=1&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E692c7bc5%2Df83b%2D4dbf%2D905d%2D7cb360d59b9e</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
-        <is>
           <t>certificados/ponentes/certificado - Segunda Elena Tolozano Benites.pdf</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
@@ -1276,15 +1225,10 @@
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>https://uniminuto0-my.sharepoint.com/personal/felix_duenas_uniminuto_edu/_layouts/15/stream.aspx?id=%2Fpersonal%2Ffelix%5Fduenas%5Funiminuto%5Fedu%2FDocuments%2FGrabaciones%2FII%20FORO%20DE%20EDITORES%20DE%20REVISTAS%20CIENT%C3%8DFICAS%2D20260911%5F080635%2DGrabaci%C3%B3n%20de%20la%20reuni%C3%B3n%2Emp4&amp;ga=1&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E692c7bc5%2Df83b%2D4dbf%2D905d%2D7cb360d59b9e</t>
-        </is>
-      </c>
-      <c r="M11" s="5" t="inlineStr">
-        <is>
           <t>certificados/ponentes/certificado - María José Orellana Tolozano.pdf</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
@@ -1348,15 +1292,10 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>https://uniminuto0-my.sharepoint.com/personal/felix_duenas_uniminuto_edu/_layouts/15/stream.aspx?id=%2Fpersonal%2Ffelix%5Fduenas%5Funiminuto%5Fedu%2FDocuments%2FGrabaciones%2FII%20FORO%20DE%20EDITORES%20DE%20REVISTAS%20CIENT%C3%8DFICAS%2D20260911%5F080635%2DGrabaci%C3%B3n%20de%20la%20reuni%C3%B3n%2Emp4&amp;ga=1&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E692c7bc5%2Df83b%2D4dbf%2D905d%2D7cb360d59b9e</t>
-        </is>
-      </c>
-      <c r="M12" s="3" t="inlineStr">
-        <is>
           <t>certificados/ponentes/certificado - Reisner de Jesús Ravelo Méndez.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
@@ -1420,15 +1359,77 @@
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>https://uniminuto0-my.sharepoint.com/personal/felix_duenas_uniminuto_edu/_layouts/15/stream.aspx?id=%2Fpersonal%2Ffelix%5Fduenas%5Funiminuto%5Fedu%2FDocuments%2FGrabaciones%2FII%20FORO%20DE%20EDITORES%20DE%20REVISTAS%20CIENT%C3%8DFICAS%2D20260911%5F080635%2DGrabaci%C3%B3n%20de%20la%20reuni%C3%B3n%2Emp4&amp;ga=1&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E692c7bc5%2Df83b%2D4dbf%2D905d%2D7cb360d59b9e</t>
-        </is>
-      </c>
-      <c r="M13" s="5" t="inlineStr">
-        <is>
           <t>certificados/ponentes/certificado - Dr. Benjamín Barón Velandia.pdf</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>FORO26-PON-013</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Leandro Ceballos Henao</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Estimado Leandro Ceballos Henao</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>juan.nieto2@utp.edu.co</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>tiflo.ceballos@gmail.com</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>C.C. 1.039.447.159</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Corporación Universitaria Minuto de Dios - UNIMINUTO</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Publicación científica para todas las personas: accesibilidad e inclusividad como criterios de calidad editorial</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Ética y buenas prácticas editoriales</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Certificado Oficial de Ponente - II Foro de Editores de Revistas Científicas 2026</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>https://juannietoval.github.io/certificaci-n-II-foro/?id=FORO26-PON-013</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>certificados/ponentes/certificado - Leandro Ceballos Henao.pdf</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>

</xml_diff>